<commit_message>
chore(config): 扩展道具表xlsx，新增 offer_in_phases 列
</commit_message>
<xml_diff>
--- a/docs/design/蛋仔--大富翁--道具表.xlsx
+++ b/docs/design/蛋仔--大富翁--道具表.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="95">
   <si>
     <t>道具id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -384,6 +384,27 @@
   <si>
     <t>使用路障卡，在你前后3格内放置一个路障，任何玩家经过此地时强制停留。</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>offer_in_phases</t>
+  </si>
+  <si>
+    <t>post_action</t>
+  </si>
+  <si>
+    <t>pre_action</t>
+  </si>
+  <si>
+    <t>pre_move</t>
+  </si>
+  <si>
+    <t>pre_action,post_action</t>
+  </si>
+  <si>
+    <t>pass_player</t>
+  </si>
+  <si>
+    <t>tax_prompt</t>
   </si>
 </sst>
 </file>
@@ -738,7 +759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="5" width="11.875" customWidth="1"/>
@@ -747,7 +768,7 @@
     <col min="10" max="10" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -781,8 +802,11 @@
       <c r="K1" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L1" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -816,8 +840,11 @@
       <c r="K2" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>2001</v>
       </c>
@@ -849,8 +876,11 @@
         <v>39</v>
       </c>
       <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L3" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2002</v>
       </c>
@@ -882,8 +912,11 @@
         <v>27</v>
       </c>
       <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>2003</v>
       </c>
@@ -915,8 +948,11 @@
         <v>31</v>
       </c>
       <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L5" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>2004</v>
       </c>
@@ -948,8 +984,11 @@
         <v>87</v>
       </c>
       <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L6" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>2005</v>
       </c>
@@ -983,8 +1022,11 @@
       <c r="K7" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L7" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>2006</v>
       </c>
@@ -1018,8 +1060,11 @@
       <c r="K8" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L8" s="1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>2007</v>
       </c>
@@ -1051,8 +1096,11 @@
         <v>84</v>
       </c>
       <c r="K9" s="1"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>2008</v>
       </c>
@@ -1084,8 +1132,11 @@
         <v>53</v>
       </c>
       <c r="K10" s="1"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>2009</v>
       </c>
@@ -1119,8 +1170,11 @@
       <c r="K11" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>2010</v>
       </c>
@@ -1152,8 +1206,11 @@
         <v>9</v>
       </c>
       <c r="K12" s="1"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>2011</v>
       </c>
@@ -1185,8 +1242,11 @@
         <v>48</v>
       </c>
       <c r="K13" s="1"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>2012</v>
       </c>
@@ -1218,8 +1278,11 @@
         <v>49</v>
       </c>
       <c r="K14" s="1"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>2013</v>
       </c>
@@ -1253,8 +1316,11 @@
       <c r="K15" s="1" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L15" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>2014</v>
       </c>
@@ -1288,8 +1354,11 @@
       <c r="K16" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>2015</v>
       </c>
@@ -1321,8 +1390,11 @@
         <v>86</v>
       </c>
       <c r="K17" s="1"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>2016</v>
       </c>
@@ -1356,8 +1428,11 @@
       <c r="K18" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>2017</v>
       </c>
@@ -1389,8 +1464,11 @@
         <v>59</v>
       </c>
       <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L19" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>2018</v>
       </c>
@@ -1422,8 +1500,11 @@
         <v>60</v>
       </c>
       <c r="K20" s="1"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>2019</v>
       </c>
@@ -1456,6 +1537,9 @@
       </c>
       <c r="K21" s="1" t="s">
         <v>61</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>